<commit_message>
Update cleaned data and adjust execution counts in cleaning notebook
</commit_message>
<xml_diff>
--- a/Aug-1/Cleaned_data.xlsx
+++ b/Aug-1/Cleaned_data.xlsx
@@ -479,7 +479,7 @@
         <v>0.1</v>
       </c>
       <c r="F2">
-        <v>134.1</v>
+        <v>121.5</v>
       </c>
       <c r="G2" s="1">
         <v>44566</v>
@@ -524,6 +524,12 @@
       <c r="D4">
         <v>60</v>
       </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>300</v>
+      </c>
       <c r="G4" s="1">
         <v>44568</v>
       </c>
@@ -548,7 +554,7 @@
         <v>0.05</v>
       </c>
       <c r="F5">
-        <v>17.03</v>
+        <v>17.081</v>
       </c>
       <c r="G5" s="1">
         <v>44569</v>
@@ -577,7 +583,7 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G6" s="1">
         <v>44743</v>
@@ -643,7 +649,7 @@
         <v>0.2</v>
       </c>
       <c r="F9">
-        <v>197.2</v>
+        <v>158.4</v>
       </c>
       <c r="G9" s="1">
         <v>44835</v>
@@ -669,7 +675,7 @@
         <v>0</v>
       </c>
       <c r="F10">
-        <v>90.5</v>
+        <v>91.5</v>
       </c>
       <c r="G10" s="1">
         <v>44572</v>
@@ -715,7 +721,7 @@
         <v>0.05</v>
       </c>
       <c r="F12">
-        <v>108.55</v>
+        <v>104.025</v>
       </c>
       <c r="G12" s="1">
         <v>44896</v>
@@ -737,6 +743,12 @@
       <c r="D13">
         <v>75</v>
       </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>150</v>
+      </c>
       <c r="G13" s="1">
         <v>44574</v>
       </c>
@@ -761,7 +773,7 @@
         <v>0</v>
       </c>
       <c r="F14">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G14" s="1">
         <v>44575</v>

</xml_diff>